<commit_message>
Expand FL connections after deep-dive on 9 unclear firms
Upgrades from UNCLEAR → YES: Bullish (Skin at Peace, West Palm Beach HQ),
Greycroft (Anine Bing / Cuyana / Goop / Madhappy — major FL retail
footprint), Maveron (Dolls Kill flagship Miami store). Upgrade from
UNCLEAR → EDGE: Mantis VC (SLUSHY, Miami HQ, adult-content caveat).
Confirmed NO after deep-dive: Cleveland Avenue, BBG Ventures, 1752vc,
Dyrdek Machine. Updated summary tab notes accordingly.

https://claude.ai/code/session_014Z9j9N5TcCLpqwigG1cFFa
</commit_message>
<xml_diff>
--- a/Magic_x_Private_Equity_Firms_FL_Highlighted.xlsx
+++ b/Magic_x_Private_Equity_Firms_FL_Highlighted.xlsx
@@ -620,12 +620,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" style="8" min="1" max="1"/>
     <col width="10" customWidth="1" style="8" min="2" max="2"/>
-    <col width="90" customWidth="1" style="8" min="3" max="3"/>
+    <col width="95" customWidth="1" style="8" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -650,7 +650,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Confirmed B2C portfolio brand HQ'd in Florida, with a major FL presence, or where FL is a top market</t>
+          <t>Confirmed B2C portfolio brand HQ'd in Florida, with a major FL operational presence, or where FL is a top market</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Borderline: B2B brand based in FL, historical/exited FL connection, or significant FL retail footprint but HQ elsewhere</t>
+          <t>Borderline: B2B brand based in FL, historical/exited FL connection, significant FL retail footprint with HQ elsewhere, or brand-safety caveat</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>Aesthetic Partners (consumer aesthetics/dermatology platform HQ in Miami, FL with multiple FL clinics)</t>
+          <t>Aesthetic Partners (consumer aesthetics/derm platform HQ in Miami, FL with multiple FL clinics)</t>
         </is>
       </c>
     </row>
@@ -786,97 +786,173 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>Skin at Peace (preservative-free skincare — HQ in West Palm Beach, FL, with manufacturing + flagship retail at Caroline Station; Bullish led rebrand and is named investment partner). Bonus: Daisy/DaisyCo (smart-home installer — HQ in CA but FL is one of two flagship markets with 7 FL service locations, the largest state footprint outside CA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Greycroft</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Multiple portfolio brands with major FL retail presence: Anine Bing (3 FL stores — Miami Design District, Aventura Mall, Sawgrass Mills); Cuyana (permanent Miami Design District store since 2019); Goop (multiple FL retail destinations — Bal Harbour/The Webster, South Beach, Design District; FL named alongside CA/TX as a top retail market); Madhappy (recurring seasonal Miami Design District shop with FL-exclusive SKUs around Art Basel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Maveron</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Dolls Kill (flagship Miami store at 2600 NW 5th Ave, Wynwood — one of only 3 US storefronts alongside LA and Las Vegas; opened March 2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Mantis Venture Capital</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>EDGE</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>SLUSHY (creator-monetization platform — HQ in Miami, FL; Mantis led $10.2M seed). NOTE: SLUSHY is an adult-content creator platform — flag for brand-safety review before treating as a usable lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>Monomoy Capital Partners</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>EDGE</t>
         </is>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C18" s="17" t="inlineStr">
         <is>
           <t>Formerly owned West Marine (2017–2021); West Marine relocated HQ to Fort Lauderdale, FL in 2022 after Monomoy exit. Also held Cast-Crete (Seffner, FL) — B2B</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>TZP Group</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>EDGE</t>
         </is>
       </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
         <is>
           <t>Palmetto Moon (apparel retailer with significant FL store footprint — Daytona, Jacksonville, Gainesville, Destin, Pensacola, Panama City Beach); Trash Butler (HQ Tampa, FL — but B2B multifamily service)</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>Gridiron Capital LLC</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>EDGE</t>
         </is>
       </c>
-      <c r="C16" s="17" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>Legacy Service Partners (HQ Tampa, FL — but B2B home services roll-up, not a consumer brand)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="18" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>Research notes</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>Research method: web search of each firm's portfolio page, Crunchbase, news releases, and press for B2C consumer brands with FL ties (HQ, major operations, or top market).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="19" t="inlineStr">
-        <is>
-          <t>Coverage gap: firms with very large portfolios (Mucker, Greycroft, Maveron, Mantis, Cleveland Avenue, Bullish, BBG Ventures, Wind Point, 1752vc, Dyrdek Machine) may contain FL-connected brands not surfaced in surface-level research. Suggest deeper portfolio review if needed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>Excluded: B2B/enterprise/SaaS investments, deep-tech, fintech infrastructure (not consumer brands).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="19" t="inlineStr">
-        <is>
-          <t>Firms confirmed NOT to have FL B2C portfolio exposure (per research): Cottonwood Technology Fund, Engage, Sageview Capital, iFly.vc, ATX Venture Partners, NuFund Venture Group, Silas Capital, Construct Capital, VestedWorld, Boathouse Capital, super{set}, Science, Alif Bank, a16z speedrun, Clocktower Ventures, Sutton Capital, HearstLab, Venrock, Modus Capital.</t>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>Methodology: Pass 1 was a full-list portfolio scan. Pass 2 was a deeper drilldown on 9 firms with large/diverse consumer portfolios (Mucker, Greycroft, Maveron, Mantis, Cleveland Avenue, Bullish, BBG Ventures, 1752vc, Dyrdek Machine) where surface-level research was inconclusive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>Pass 2 upgrades (UNCLEAR → YES): Bullish (Skin at Peace), Greycroft (Anine Bing, Cuyana, Goop, Madhappy), Maveron (Dolls Kill). Pass 2 upgrade (UNCLEAR → EDGE): Mantis VC (SLUSHY, with adult-content brand-safety caveat).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>Confirmed NO after deep-dive: Cleveland Avenue, BBG Ventures, 1752vc/Pegasus, Dyrdek Machine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>Mucker Capital: portfolio of 60+ consumer companies could not be fully enumerated from public sources (portfolio page + Crunchbase/PitchBook/CBInsights blocked). Brands that were surfaced are all CA-HQ'd. Recommend a paid PitchBook/Crunchbase export filtered by investor + portfolio HQ state = FL for full coverage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>Other firms confirmed NO from Pass 1: Cottonwood Technology Fund, Engage, Sageview Capital, iFly.vc, ATX Venture Partners, NuFund Venture Group, Silas Capital, Construct Capital, VestedWorld, Boathouse Capital, super{set}, Science, Alif Bank, a16z speedrun, Clocktower Ventures, Sutton Capital, HearstLab, Venrock, Modus Capital.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A22:C22"/>
+  <mergeCells count="5">
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A24:C24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -901,7 +977,7 @@
     <col width="14.5546875" bestFit="1" customWidth="1" style="4" min="9" max="9"/>
     <col width="21" bestFit="1" customWidth="1" style="4" min="10" max="10"/>
     <col width="20" customWidth="1" style="8" min="11" max="11"/>
-    <col width="80" customWidth="1" style="8" min="12" max="12"/>
+    <col width="90" customWidth="1" style="8" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -963,47 +1039,55 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="21" t="inlineStr">
         <is>
           <t>Bullish</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>San Francisco, CA</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="22" t="inlineStr">
         <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="E3" s="20" t="n">
+      <c r="E3" s="23" t="n">
         <v>20809000000</v>
       </c>
-      <c r="F3" s="20" t="n">
+      <c r="F3" s="23" t="n">
         <v>244811400000</v>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="24" t="inlineStr">
         <is>
           <t>9.8</t>
         </is>
       </c>
-      <c r="H3" s="20" t="n">
+      <c r="H3" s="23" t="n">
         <v>21200000</v>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="22" t="inlineStr">
         <is>
           <t>414</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>46.8%</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="K3" s="12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L3" s="15" t="inlineStr">
+        <is>
+          <t>Skin at Peace (preservative-free skincare — HQ in West Palm Beach, FL, with manufacturing + flagship retail at Caroline Station; Bullish led rebrand and is named investment partner). Bonus: Daisy/DaisyCo (smart-home installer — HQ in CA but FL is one of two flagship markets with 7 FL service locations, the largest state footprint outside CA)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="B4" s="7" t="inlineStr">
@@ -1045,8 +1129,6 @@
           <t>13.3%</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="B5" s="7" t="inlineStr">
@@ -1088,8 +1170,6 @@
           <t>13.7%</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="B6" s="7" t="inlineStr">
@@ -1125,8 +1205,6 @@
           <t>95.0%</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="7" t="inlineStr">
@@ -1166,8 +1244,6 @@
           <t>3.9%</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="B8" s="7" t="inlineStr">
@@ -1205,8 +1281,6 @@
       <c r="J8" s="9" t="n">
         <v>-0.015</v>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="B9" s="7" t="inlineStr">
@@ -1248,8 +1322,6 @@
           <t>10.4%</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="B10" s="7" t="inlineStr">
@@ -1289,8 +1361,6 @@
       <c r="J10" s="9" t="n">
         <v>-0.471</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="B11" s="7" t="inlineStr">
@@ -1330,8 +1400,6 @@
           <t>13.2%</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="B12" s="21" t="inlineStr">
@@ -1422,8 +1490,6 @@
       <c r="J13" s="9" t="n">
         <v>-0.306</v>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="7" t="inlineStr">
@@ -1465,8 +1531,6 @@
           <t>28.6%</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="B15" s="21" t="inlineStr">
@@ -1606,8 +1670,6 @@
           <t>7.4%</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="B18" s="7" t="inlineStr">
@@ -1649,8 +1711,6 @@
           <t>3.8%</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="B19" s="7" t="inlineStr">
@@ -1690,8 +1750,6 @@
       <c r="J19" s="9" t="n">
         <v>-0.014</v>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="B20" s="7" t="inlineStr">
@@ -1731,47 +1789,53 @@
           <t>5.4%</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="26" t="inlineStr">
         <is>
           <t>Mantis Venture Capital</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="16" t="inlineStr">
         <is>
           <t>Los Angeles, CA</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="27" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="E21" s="20" t="n">
+      <c r="E21" s="28" t="n">
         <v>712781</v>
       </c>
-      <c r="F21" s="20" t="n">
+      <c r="F21" s="28" t="n">
         <v>8385657</v>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="G21" s="29" t="inlineStr">
         <is>
           <t>8.8</t>
         </is>
       </c>
-      <c r="H21" s="20" t="n">
+      <c r="H21" s="28" t="n">
         <v>135000000</v>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="I21" s="27" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
+      <c r="J21" s="27" t="inlineStr"/>
+      <c r="K21" s="13" t="inlineStr">
+        <is>
+          <t>EDGE</t>
+        </is>
+      </c>
+      <c r="L21" s="17" t="inlineStr">
+        <is>
+          <t>SLUSHY (creator-monetization platform — HQ in Miami, FL; Mantis led $10.2M seed). NOTE: SLUSHY is an adult-content creator platform — flag for brand-safety review before treating as a usable lead</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="B22" s="21" t="inlineStr">
@@ -1871,50 +1935,58 @@
       </c>
       <c r="L23" s="15" t="inlineStr">
         <is>
-          <t>Aesthetic Partners (consumer aesthetics/dermatology platform HQ in Miami, FL with multiple FL clinics)</t>
+          <t>Aesthetic Partners (consumer aesthetics/derm platform HQ in Miami, FL with multiple FL clinics)</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="21" t="inlineStr">
         <is>
           <t>Greycroft</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="22" t="inlineStr">
         <is>
           <t>2006</t>
         </is>
       </c>
-      <c r="E24" s="20" t="n">
+      <c r="E24" s="23" t="n">
         <v>2656729</v>
       </c>
-      <c r="F24" s="20" t="n">
+      <c r="F24" s="23" t="n">
         <v>31255632</v>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="24" t="inlineStr">
         <is>
           <t>9.8</t>
         </is>
       </c>
-      <c r="H24" s="20" t="n">
+      <c r="H24" s="23" t="n">
         <v>2288600000</v>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="I24" s="22" t="inlineStr">
         <is>
           <t>82</t>
         </is>
       </c>
-      <c r="J24" s="9" t="n">
+      <c r="J24" s="25" t="n">
         <v>-0.035</v>
       </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
+      <c r="K24" s="12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L24" s="15" t="inlineStr">
+        <is>
+          <t>Multiple portfolio brands with major FL retail presence: Anine Bing (3 FL stores — Miami Design District, Aventura Mall, Sawgrass Mills); Cuyana (permanent Miami Design District store since 2019); Goop (multiple FL retail destinations — Bal Harbour/The Webster, South Beach, Design District; FL named alongside CA/TX as a top retail market); Madhappy (recurring seasonal Miami Design District shop with FL-exclusive SKUs around Art Basel)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="26" t="inlineStr">
@@ -2003,8 +2075,6 @@
           <t>6.3%</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="B27" s="7" t="inlineStr">
@@ -2044,8 +2114,6 @@
       <c r="J27" s="9" t="n">
         <v>-0.044</v>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="B28" s="7" t="inlineStr">
@@ -2081,47 +2149,53 @@
           <t>22.7%</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B29" s="21" t="inlineStr">
         <is>
           <t>Maveron</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>San Francisco, CA</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="22" t="inlineStr">
         <is>
           <t>1998</t>
         </is>
       </c>
-      <c r="E29" s="20" t="n">
+      <c r="E29" s="23" t="n">
         <v>680382</v>
       </c>
-      <c r="F29" s="20" t="n">
+      <c r="F29" s="23" t="n">
         <v>8004491</v>
       </c>
-      <c r="G29" s="6" t="inlineStr"/>
-      <c r="H29" s="20" t="n">
+      <c r="G29" s="24" t="inlineStr"/>
+      <c r="H29" s="23" t="n">
         <v>247725000</v>
       </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="I29" s="22" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="J29" s="22" t="inlineStr">
         <is>
           <t>5.0%</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+      <c r="K29" s="12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L29" s="15" t="inlineStr">
+        <is>
+          <t>Dolls Kill (flagship Miami store at 2600 NW 5th Ave, Wynwood — one of only 3 US storefronts alongside LA and Las Vegas; opened March 2025)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="7" t="inlineStr">
@@ -2163,8 +2237,6 @@
           <t>2.5%</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="B31" s="7" t="inlineStr">
@@ -2206,8 +2278,6 @@
           <t>50.0%</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="B32" s="7" t="inlineStr">
@@ -2249,8 +2319,6 @@
           <t>17.9%</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="B33" s="7" t="inlineStr">
@@ -2292,8 +2360,6 @@
           <t>6.7%</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="B34" s="7" t="inlineStr">
@@ -2335,8 +2401,6 @@
           <t>6.3%</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="B35" s="7" t="inlineStr">
@@ -2376,8 +2440,6 @@
       <c r="J35" s="9" t="n">
         <v>-0.227</v>
       </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="B36" s="7" t="inlineStr">
@@ -2417,8 +2479,6 @@
       <c r="J36" s="9" t="n">
         <v>-0.167</v>
       </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="B37" s="26" t="inlineStr">
@@ -2511,8 +2571,6 @@
       <c r="J38" s="9" t="n">
         <v>-0.167</v>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="B39" s="26" t="inlineStr">
@@ -2597,8 +2655,6 @@
       <c r="J40" s="9" t="n">
         <v>-0.154</v>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="B41" s="21" t="inlineStr">
@@ -2685,8 +2741,6 @@
           <t>10.0%</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="B43" s="7" t="inlineStr">
@@ -2722,8 +2776,6 @@
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="B44" s="7" t="inlineStr">
@@ -2759,8 +2811,6 @@
       <c r="J44" s="9" t="n">
         <v>-0.2</v>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="B45" s="7" t="inlineStr">
@@ -2798,8 +2848,6 @@
           <t>9.5%</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="B46" s="7" t="inlineStr">
@@ -2839,8 +2887,6 @@
       <c r="J46" s="9" t="n">
         <v>-0.188</v>
       </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="B47" s="7" t="inlineStr">
@@ -2882,8 +2928,6 @@
           <t>12.9%</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="B48" s="7" t="inlineStr">
@@ -2919,8 +2963,6 @@
           <t>4.5%</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="B49" s="7" t="inlineStr">
@@ -2962,8 +3004,6 @@
           <t>7.1%</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="B50" s="7" t="inlineStr">
@@ -3005,8 +3045,6 @@
           <t>18.7%</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="B51" s="7" t="inlineStr">
@@ -3048,8 +3086,6 @@
           <t>11.4%</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>